<commit_message>
Enhance player model to include appointment requests and update scheduling logic to consider daily requests; modify Excel template for improved layout and clarity.
</commit_message>
<xml_diff>
--- a/templates/planning_template.xlsx
+++ b/templates/planning_template.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Planning" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Schedule" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -56,8 +56,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -426,362 +429,941 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B49"/>
+  <dimension ref="A1:N51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Horaire</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
+          <t>Monday</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Thursday</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Pseudo</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>00:15</t>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Trigram</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Pseudo</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Trigram</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Pseudo</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Trigram</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>ID</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>00:45</t>
+          <t>23:45 (veille)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>23:45 (veille)</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>23:45 (veille)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>01:15</t>
+          <t>00:15</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>00:15</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>00:15</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>01:45</t>
+          <t>00:45</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>00:45</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>00:45</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>02:15</t>
+          <t>01:15</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>01:15</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>01:15</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>02:45</t>
+          <t>01:45</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>01:45</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>01:45</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>03:15</t>
+          <t>02:15</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>02:15</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>02:15</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>03:45</t>
+          <t>02:45</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>02:45</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>02:45</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>04:15</t>
+          <t>03:15</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>03:15</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>03:15</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>04:45</t>
+          <t>03:45</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>03:45</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>03:45</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05:15</t>
+          <t>04:15</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>04:15</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>04:15</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>05:45</t>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>04:45</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>04:45</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>06:15</t>
+          <t>05:15</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>05:15</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>05:15</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>06:45</t>
+          <t>05:45</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>05:45</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>05:45</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>07:15</t>
+          <t>06:15</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>06:15</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>06:15</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07:45</t>
+          <t>06:45</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>06:45</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>06:45</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08:15</t>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>07:15</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>07:15</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>08:45</t>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>07:45</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>07:45</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>08:15</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>08:45</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>09:15</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>10:45</t>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>09:45</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>10:15</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>10:45</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>11:15</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>11:15</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>11:45</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>13:15</t>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>12:15</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>12:45</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>14:15</t>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>13:15</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>14:45</t>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>13:45</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>15:15</t>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>14:15</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>14:15</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>15:45</t>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>14:45</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>16:15</t>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>15:15</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>16:45</t>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>15:45</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>17:15</t>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>16:15</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>17:45</t>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>16:45</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>18:15</t>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>17:15</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>18:45</t>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>17:45</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>17:45</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>19:15</t>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>18:15</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>18:15</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>19:45</t>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>18:45</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>20:15</t>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>19:15</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>20:45</t>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>19:45</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>21:15</t>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>20:15</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>20:15</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>21:45</t>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>20:45</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>20:45</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>22:15</t>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>21:15</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>21:15</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>22:45</t>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>21:45</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>21:45</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>23:15</t>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>22:15</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>22:15</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
+          <t>22:45</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>22:45</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>22:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>23:15</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>23:15</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
           <t>23:45</t>
         </is>
       </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>23:45</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>23:45</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="K1:N1"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="F1:I1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>